<commit_message>
Add enriching KG script. Update data file.
</commit_message>
<xml_diff>
--- a/Data/NiSuperAlloyProperties.xlsx
+++ b/Data/NiSuperAlloyProperties.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="222">
   <si>
     <t>Alloy</t>
   </si>
@@ -51,7 +51,7 @@
     <t>Inconel 600</t>
   </si>
   <si>
-    <t>≥72.0</t>
+    <t>&gt;=72.0</t>
   </si>
   <si>
     <t>14.0-17.0</t>
@@ -63,7 +63,7 @@
     <t>6.0-10.0</t>
   </si>
   <si>
-    <t>Cu ≤0.5</t>
+    <t>Cu&lt;=0.5</t>
   </si>
   <si>
     <t>Inconel 617</t>
@@ -84,28 +84,28 @@
     <t>0.8-1.5</t>
   </si>
   <si>
-    <t>≤0.6</t>
-  </si>
-  <si>
-    <t>≤3.0</t>
+    <t>&lt;=0.6</t>
+  </si>
+  <si>
+    <t>&lt;=3.0</t>
   </si>
   <si>
     <t>Inconel 625</t>
   </si>
   <si>
-    <t>≥58.0</t>
+    <t>&gt;=58.0</t>
   </si>
   <si>
     <t>20.0-23.0</t>
   </si>
   <si>
-    <t>≤1.0</t>
-  </si>
-  <si>
-    <t>≤0.4</t>
-  </si>
-  <si>
-    <t>≤5.0</t>
+    <t>&lt;=1.0</t>
+  </si>
+  <si>
+    <t>&lt;=0.4</t>
+  </si>
+  <si>
+    <t>&lt;=5.0</t>
   </si>
   <si>
     <t>3.15-4.15</t>
@@ -129,19 +129,19 @@
     <t>0.65-1.15</t>
   </si>
   <si>
-    <t>Bal.</t>
+    <t>BAL</t>
   </si>
   <si>
     <t>4.75-5.5</t>
   </si>
   <si>
-    <t>B ≤0.006</t>
+    <t>B&lt;=0.006</t>
   </si>
   <si>
     <t>Inconel X-750</t>
   </si>
   <si>
-    <t>≥70.0</t>
+    <t>&gt;=70.0</t>
   </si>
   <si>
     <t>0.4-1.0</t>
@@ -165,16 +165,16 @@
     <t>19.0-23.0</t>
   </si>
   <si>
-    <t>≤0.15</t>
+    <t>&lt;=0.15</t>
   </si>
   <si>
     <t>0.15-0.6</t>
   </si>
   <si>
-    <t>≥39.5</t>
-  </si>
-  <si>
-    <t>Cu ≤0.75</t>
+    <t>&gt;=39.5</t>
+  </si>
+  <si>
+    <t>Cu&lt;=0.75</t>
   </si>
   <si>
     <t>Inconel 825</t>
@@ -189,13 +189,13 @@
     <t>2.5-3.5</t>
   </si>
   <si>
-    <t>≤0.2</t>
+    <t>&lt;=0.2</t>
   </si>
   <si>
     <t>0.6-1.2</t>
   </si>
   <si>
-    <t>≥22.0</t>
+    <t>&gt;=22.0</t>
   </si>
   <si>
     <t>Cu 1.5-3.0</t>
@@ -222,13 +222,13 @@
     <t>Hastelloy C-276</t>
   </si>
   <si>
-    <t>≥52.0</t>
+    <t>&gt;=52.0</t>
   </si>
   <si>
     <t>14.5-16.5</t>
   </si>
   <si>
-    <t>≤2.5</t>
+    <t>&lt;=2.5</t>
   </si>
   <si>
     <t>15.0-17.0</t>
@@ -240,7 +240,7 @@
     <t>4.0-7.0</t>
   </si>
   <si>
-    <t>V ≤0.35</t>
+    <t>V&lt;=0.35</t>
   </si>
   <si>
     <t>Waspaloy</t>
@@ -261,10 +261,10 @@
     <t>2.75-3.25</t>
   </si>
   <si>
-    <t>≤2.0</t>
-  </si>
-  <si>
-    <t>Zr ≤0.07</t>
+    <t>&lt;=2.0</t>
+  </si>
+  <si>
+    <t>Zr&lt;=0.07</t>
   </si>
   <si>
     <t>Rene 41</t>
@@ -285,7 +285,7 @@
     <t>3.0-3.5</t>
   </si>
   <si>
-    <t>B ≤0.005</t>
+    <t>B&lt;=0.005</t>
   </si>
   <si>
     <t>Rene 88DT</t>
@@ -303,7 +303,7 @@
     <t>3.2-3.8</t>
   </si>
   <si>
-    <t>Zr ≤0.03</t>
+    <t>Zr&lt;=0.03</t>
   </si>
   <si>
     <t>Haynes 230</t>
@@ -318,10 +318,10 @@
     <t>0.2-0.5</t>
   </si>
   <si>
-    <t>≤0.1</t>
-  </si>
-  <si>
-    <t>La ≤0.02</t>
+    <t>&lt;=0.1</t>
+  </si>
+  <si>
+    <t>La&lt;=0.02</t>
   </si>
   <si>
     <t>Haynes 282</t>
@@ -342,7 +342,7 @@
     <t>2.0-2.4</t>
   </si>
   <si>
-    <t>≤1.5</t>
+    <t>&lt;=1.5</t>
   </si>
   <si>
     <t>Nimonic 80A</t>
@@ -372,10 +372,10 @@
     <t>2.5-3.3</t>
   </si>
   <si>
-    <t>≤4.0</t>
-  </si>
-  <si>
-    <t>B ≤0.015</t>
+    <t>&lt;=4.0</t>
+  </si>
+  <si>
+    <t>B&lt;=0.015</t>
   </si>
   <si>
     <t>Udimet 720</t>
@@ -417,7 +417,7 @@
     <t>0.8-1.2</t>
   </si>
   <si>
-    <t>≤0.5</t>
+    <t>&lt;=0.5</t>
   </si>
   <si>
     <t>Re 2.8-3.2</t>
@@ -438,243 +438,181 @@
     <t>Elastic Modulus (E, GPa)</t>
   </si>
   <si>
-    <t>550–620</t>
-  </si>
-  <si>
-    <t>240–415</t>
-  </si>
-  <si>
-    <t>30–55</t>
-  </si>
-  <si>
-    <t>B75–B90</t>
+    <t>550-620</t>
+  </si>
+  <si>
+    <t>240-415</t>
+  </si>
+  <si>
+    <t>30-55</t>
+  </si>
+  <si>
+    <t>HRB75-90</t>
   </si>
   <si>
     <t>~205</t>
   </si>
   <si>
-    <t>760–950</t>
-  </si>
-  <si>
-    <t>380–550</t>
-  </si>
-  <si>
-    <t>30–50</t>
-  </si>
-  <si>
-    <t>B85–B95</t>
-  </si>
-  <si>
-    <t>930–1030</t>
-  </si>
-  <si>
-    <t>517–725</t>
-  </si>
-  <si>
-    <t>30–45</t>
-  </si>
-  <si>
-    <t>B96–B100</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">~207 (GPa) </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>Wikipedia</t>
-    </r>
-  </si>
-  <si>
-    <t>1240–1430</t>
-  </si>
-  <si>
-    <t>1030–1170</t>
-  </si>
-  <si>
-    <t>12–25</t>
-  </si>
-  <si>
-    <t>C35–C45</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">~208 (GPa) </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>hightempmetals.com</t>
-    </r>
-  </si>
-  <si>
-    <t>Inconel X‑750</t>
-  </si>
-  <si>
-    <t>C35</t>
-  </si>
-  <si>
-    <t>500–650</t>
-  </si>
-  <si>
-    <t>200–300</t>
-  </si>
-  <si>
-    <t>B75–B85</t>
-  </si>
-  <si>
-    <t>586–690</t>
-  </si>
-  <si>
-    <t>241–345</t>
-  </si>
-  <si>
-    <t>690–760</t>
-  </si>
-  <si>
-    <t>310–350</t>
-  </si>
-  <si>
-    <t>35–50</t>
-  </si>
-  <si>
-    <t>Hastelloy C‑276</t>
-  </si>
-  <si>
-    <t>790–900</t>
-  </si>
-  <si>
-    <t>415–550</t>
-  </si>
-  <si>
-    <t>40–60</t>
-  </si>
-  <si>
-    <t>B90–B100</t>
-  </si>
-  <si>
-    <t>1200–1350</t>
-  </si>
-  <si>
-    <t>800–950</t>
-  </si>
-  <si>
-    <t>15–25</t>
-  </si>
-  <si>
-    <t>C35–C40</t>
-  </si>
-  <si>
-    <t>1450–1600</t>
-  </si>
-  <si>
-    <t>1000–1200</t>
-  </si>
-  <si>
-    <t>10–20</t>
-  </si>
-  <si>
-    <t>C40–C45</t>
-  </si>
-  <si>
-    <t>1400–1550</t>
-  </si>
-  <si>
-    <t>950–1100</t>
-  </si>
-  <si>
-    <t>12–18</t>
-  </si>
-  <si>
-    <t>C38–C42</t>
-  </si>
-  <si>
-    <t>760–900</t>
-  </si>
-  <si>
-    <t>350–450</t>
-  </si>
-  <si>
-    <t>40–55</t>
-  </si>
-  <si>
-    <t>1000–1150</t>
-  </si>
-  <si>
-    <t>700–850</t>
-  </si>
-  <si>
-    <t>C30–C40</t>
-  </si>
-  <si>
-    <t>1100–1300</t>
-  </si>
-  <si>
-    <t>750–900</t>
-  </si>
-  <si>
-    <t>1300–1500</t>
-  </si>
-  <si>
-    <t>900–1100</t>
-  </si>
-  <si>
-    <t>1400–1600</t>
-  </si>
-  <si>
-    <t>10–15</t>
-  </si>
-  <si>
-    <t>C42–C48</t>
-  </si>
-  <si>
-    <t>Mar‑M247 (cast)</t>
-  </si>
-  <si>
-    <t>5–10</t>
-  </si>
-  <si>
-    <t>CMSX‑4 (single‑crystal)</t>
-  </si>
-  <si>
-    <t>1350–1500</t>
-  </si>
-  <si>
-    <t>8–15</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">~205 (macroscopic average); single‑crystal directions vary widely between ~138 GPa and ~241 GPa along different crystal axes </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>Nature</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-      </rPr>
-      <t/>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>MDPI</t>
-    </r>
+    <t>760-950</t>
+  </si>
+  <si>
+    <t>380-550</t>
+  </si>
+  <si>
+    <t>30-50</t>
+  </si>
+  <si>
+    <t>HRB85-95</t>
+  </si>
+  <si>
+    <t>930-1030</t>
+  </si>
+  <si>
+    <t>517-725</t>
+  </si>
+  <si>
+    <t>30-45</t>
+  </si>
+  <si>
+    <t>HRB96-100</t>
+  </si>
+  <si>
+    <t>~207</t>
+  </si>
+  <si>
+    <t>1240-1430</t>
+  </si>
+  <si>
+    <t>1030-1170</t>
+  </si>
+  <si>
+    <t>12-25</t>
+  </si>
+  <si>
+    <t>HRC35-45</t>
+  </si>
+  <si>
+    <t>~208</t>
+  </si>
+  <si>
+    <t>HRC35</t>
+  </si>
+  <si>
+    <t>500-650</t>
+  </si>
+  <si>
+    <t>200-300</t>
+  </si>
+  <si>
+    <t>HRB75-85</t>
+  </si>
+  <si>
+    <t>586-690</t>
+  </si>
+  <si>
+    <t>241-345</t>
+  </si>
+  <si>
+    <t>690-760</t>
+  </si>
+  <si>
+    <t>310-350</t>
+  </si>
+  <si>
+    <t>35-50</t>
+  </si>
+  <si>
+    <t>790-900</t>
+  </si>
+  <si>
+    <t>415-550</t>
+  </si>
+  <si>
+    <t>40-60</t>
+  </si>
+  <si>
+    <t>HRB90-100</t>
+  </si>
+  <si>
+    <t>1200-1350</t>
+  </si>
+  <si>
+    <t>800-950</t>
+  </si>
+  <si>
+    <t>15-25</t>
+  </si>
+  <si>
+    <t>HRC35-40</t>
+  </si>
+  <si>
+    <t>1450-1600</t>
+  </si>
+  <si>
+    <t>1000-1200</t>
+  </si>
+  <si>
+    <t>10-20</t>
+  </si>
+  <si>
+    <t>HRC40-45</t>
+  </si>
+  <si>
+    <t>1400-1550</t>
+  </si>
+  <si>
+    <t>950-1100</t>
+  </si>
+  <si>
+    <t>12-18</t>
+  </si>
+  <si>
+    <t>HRC38-42</t>
+  </si>
+  <si>
+    <t>760-900</t>
+  </si>
+  <si>
+    <t>350-450</t>
+  </si>
+  <si>
+    <t>40-55</t>
+  </si>
+  <si>
+    <t>1000-1150</t>
+  </si>
+  <si>
+    <t>700-850</t>
+  </si>
+  <si>
+    <t>HRC30-40</t>
+  </si>
+  <si>
+    <t>1100-1300</t>
+  </si>
+  <si>
+    <t>750-900</t>
+  </si>
+  <si>
+    <t>1300-1500</t>
+  </si>
+  <si>
+    <t>900-1100</t>
+  </si>
+  <si>
+    <t>1400-1600</t>
+  </si>
+  <si>
+    <t>10-15</t>
+  </si>
+  <si>
+    <t>HRC42-48</t>
+  </si>
+  <si>
+    <t>1350-1500</t>
+  </si>
+  <si>
+    <t>8-15</t>
   </si>
   <si>
     <t>Density (g/cm³)</t>
@@ -747,6 +685,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="d-m"/>
+  </numFmts>
   <fonts count="5">
     <font>
       <sz val="10.0"/>
@@ -767,10 +708,10 @@
     <font>
       <color theme="1"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <color rgb="FF0000FF"/>
+      <color theme="1"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -804,7 +745,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -815,16 +756,19 @@
       <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
+      <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="2" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right" vertical="bottom"/>
@@ -1816,61 +1760,62 @@
       <c r="F1" s="3" t="s">
         <v>140</v>
       </c>
+      <c r="G1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="5" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="5" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>153</v>
       </c>
       <c r="F4" s="5" t="s">
@@ -1878,19 +1823,19 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>158</v>
       </c>
       <c r="F5" s="5" t="s">
@@ -1898,8 +1843,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="s">
-        <v>160</v>
+      <c r="A6" s="5" t="s">
+        <v>41</v>
       </c>
       <c r="B6" s="6">
         <v>1260.0</v>
@@ -1910,320 +1855,315 @@
       <c r="D6" s="6">
         <v>20.0</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="C7" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="D7" s="4" t="s">
+    <row r="8">
+      <c r="A8" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="F7" s="4" t="s">
+      <c r="E8" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="C8" s="4" t="s">
+    <row r="9">
+      <c r="A9" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="E8" s="4" t="s">
+      <c r="C9" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F9" s="5" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="D9" s="4" t="s">
+    <row r="10">
+      <c r="A10" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="C10" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F14" s="5" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="E10" s="4" t="s">
+    <row r="15">
+      <c r="A15" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="D20" s="7">
+        <v>45935.0</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="F20" s="5" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="E11" s="4" t="s">
+    <row r="21">
+      <c r="A21" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="D21" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="F21" s="5" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>205</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink r:id="rId1" ref="F4"/>
-    <hyperlink r:id="rId2" ref="F5"/>
-    <hyperlink r:id="rId3" ref="F21"/>
-  </hyperlinks>
-  <drawing r:id="rId4"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2239,38 +2179,38 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="7">
+      <c r="B2" s="8">
         <v>8.47</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="D2" s="7">
+        <v>205</v>
+      </c>
+      <c r="D2" s="8">
         <v>14.9</v>
       </c>
-      <c r="E2" s="7">
+      <c r="E2" s="8">
         <v>13.3</v>
       </c>
-      <c r="F2" s="7">
+      <c r="F2" s="8">
         <v>1.03</v>
       </c>
     </row>
@@ -2278,19 +2218,19 @@
       <c r="A3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="8">
         <v>8.36</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="D3" s="7">
+        <v>206</v>
+      </c>
+      <c r="D3" s="8">
         <v>11.7</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="8">
         <v>12.5</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="8">
         <v>1.25</v>
       </c>
     </row>
@@ -2298,19 +2238,19 @@
       <c r="A4" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="8">
         <v>8.44</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="D4" s="7">
+        <v>207</v>
+      </c>
+      <c r="D4" s="8">
         <v>9.8</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="8">
         <v>12.8</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="8">
         <v>1.28</v>
       </c>
     </row>
@@ -2318,19 +2258,19 @@
       <c r="A5" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="8">
         <v>8.19</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="D5" s="7">
+        <v>208</v>
+      </c>
+      <c r="D5" s="8">
         <v>11.4</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="8">
         <v>11.8</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="8">
         <v>1.25</v>
       </c>
     </row>
@@ -2338,19 +2278,19 @@
       <c r="A6" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="8">
         <v>8.28</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="D6" s="7">
+        <v>209</v>
+      </c>
+      <c r="D6" s="8">
         <v>11.7</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="8">
         <v>13.3</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="8">
         <v>1.22</v>
       </c>
     </row>
@@ -2358,19 +2298,19 @@
       <c r="A7" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="8">
         <v>7.94</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="D7" s="7">
+        <v>210</v>
+      </c>
+      <c r="D7" s="8">
         <v>11.8</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="8">
         <v>14.4</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="8">
         <v>0.98</v>
       </c>
     </row>
@@ -2378,19 +2318,19 @@
       <c r="A8" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="8">
         <v>8.14</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="D8" s="7">
+        <v>211</v>
+      </c>
+      <c r="D8" s="8">
         <v>10.9</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="8">
         <v>14.0</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="8">
         <v>1.15</v>
       </c>
     </row>
@@ -2398,19 +2338,19 @@
       <c r="A9" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="8">
         <v>8.22</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="D9" s="7">
+        <v>212</v>
+      </c>
+      <c r="D9" s="8">
         <v>9.8</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="8">
         <v>14.0</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="8">
         <v>1.2</v>
       </c>
     </row>
@@ -2418,19 +2358,19 @@
       <c r="A10" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="8">
         <v>8.89</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="D10" s="7">
+        <v>213</v>
+      </c>
+      <c r="D10" s="8">
         <v>10.1</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="8">
         <v>12.6</v>
       </c>
-      <c r="F10" s="7">
+      <c r="F10" s="8">
         <v>1.3</v>
       </c>
     </row>
@@ -2438,19 +2378,19 @@
       <c r="A11" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B11" s="7">
+      <c r="B11" s="8">
         <v>8.22</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="D11" s="7">
+        <v>206</v>
+      </c>
+      <c r="D11" s="8">
         <v>11.0</v>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="8">
         <v>12.5</v>
       </c>
-      <c r="F11" s="7">
+      <c r="F11" s="8">
         <v>1.25</v>
       </c>
     </row>
@@ -2458,19 +2398,19 @@
       <c r="A12" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12" s="8">
         <v>8.27</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="D12" s="7">
+        <v>214</v>
+      </c>
+      <c r="D12" s="8">
         <v>10.5</v>
       </c>
-      <c r="E12" s="7">
+      <c r="E12" s="8">
         <v>12.0</v>
       </c>
-      <c r="F12" s="7">
+      <c r="F12" s="8">
         <v>1.3</v>
       </c>
     </row>
@@ -2478,19 +2418,19 @@
       <c r="A13" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B13" s="7">
+      <c r="B13" s="8">
         <v>8.2</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="D13" s="7">
+        <v>215</v>
+      </c>
+      <c r="D13" s="8">
         <v>10.8</v>
       </c>
-      <c r="E13" s="7">
+      <c r="E13" s="8">
         <v>11.8</v>
       </c>
-      <c r="F13" s="7">
+      <c r="F13" s="8">
         <v>1.28</v>
       </c>
     </row>
@@ -2498,19 +2438,19 @@
       <c r="A14" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B14" s="7">
+      <c r="B14" s="8">
         <v>8.97</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="D14" s="7">
+        <v>214</v>
+      </c>
+      <c r="D14" s="8">
         <v>11.1</v>
       </c>
-      <c r="E14" s="7">
+      <c r="E14" s="8">
         <v>12.5</v>
       </c>
-      <c r="F14" s="7">
+      <c r="F14" s="8">
         <v>1.22</v>
       </c>
     </row>
@@ -2518,19 +2458,19 @@
       <c r="A15" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B15" s="7">
+      <c r="B15" s="8">
         <v>8.25</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="D15" s="7">
+        <v>216</v>
+      </c>
+      <c r="D15" s="8">
         <v>10.5</v>
       </c>
-      <c r="E15" s="7">
+      <c r="E15" s="8">
         <v>12.0</v>
       </c>
-      <c r="F15" s="7">
+      <c r="F15" s="8">
         <v>1.3</v>
       </c>
     </row>
@@ -2538,19 +2478,19 @@
       <c r="A16" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B16" s="7">
+      <c r="B16" s="8">
         <v>8.19</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="D16" s="7">
+        <v>217</v>
+      </c>
+      <c r="D16" s="8">
         <v>11.0</v>
       </c>
-      <c r="E16" s="7">
+      <c r="E16" s="8">
         <v>12.5</v>
       </c>
-      <c r="F16" s="7">
+      <c r="F16" s="8">
         <v>1.25</v>
       </c>
     </row>
@@ -2558,19 +2498,19 @@
       <c r="A17" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B17" s="7">
+      <c r="B17" s="8">
         <v>8.2</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="D17" s="7">
+        <v>214</v>
+      </c>
+      <c r="D17" s="8">
         <v>10.8</v>
       </c>
-      <c r="E17" s="7">
+      <c r="E17" s="8">
         <v>12.0</v>
       </c>
-      <c r="F17" s="7">
+      <c r="F17" s="8">
         <v>1.28</v>
       </c>
     </row>
@@ -2578,19 +2518,19 @@
       <c r="A18" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B18" s="7">
+      <c r="B18" s="8">
         <v>8.22</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="D18" s="7">
+        <v>218</v>
+      </c>
+      <c r="D18" s="8">
         <v>10.5</v>
       </c>
-      <c r="E18" s="7">
+      <c r="E18" s="8">
         <v>12.5</v>
       </c>
-      <c r="F18" s="7">
+      <c r="F18" s="8">
         <v>1.3</v>
       </c>
     </row>
@@ -2598,19 +2538,19 @@
       <c r="A19" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="B19" s="7">
+      <c r="B19" s="8">
         <v>8.25</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="D19" s="7">
+        <v>219</v>
+      </c>
+      <c r="D19" s="8">
         <v>10.0</v>
       </c>
-      <c r="E19" s="7">
+      <c r="E19" s="8">
         <v>12.0</v>
       </c>
-      <c r="F19" s="7">
+      <c r="F19" s="8">
         <v>1.35</v>
       </c>
     </row>
@@ -2618,39 +2558,39 @@
       <c r="A20" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B20" s="7">
+      <c r="B20" s="8">
         <v>8.9</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="D20" s="7">
+        <v>220</v>
+      </c>
+      <c r="D20" s="8">
         <v>9.5</v>
       </c>
-      <c r="E20" s="7">
+      <c r="E20" s="8">
         <v>11.5</v>
       </c>
-      <c r="F20" s="7">
+      <c r="F20" s="8">
         <v>1.4</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="B21" s="7">
+        <v>221</v>
+      </c>
+      <c r="B21" s="8">
         <v>8.7</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="D21" s="7">
+        <v>217</v>
+      </c>
+      <c r="D21" s="8">
         <v>9.0</v>
       </c>
-      <c r="E21" s="7">
+      <c r="E21" s="8">
         <v>11.0</v>
       </c>
-      <c r="F21" s="7">
+      <c r="F21" s="8">
         <v>1.45</v>
       </c>
     </row>

</xml_diff>